<commit_message>
template: the piezo sheet's 'Type options' header spelled right, and no stray space before 'Phreatic surface' (owner 163 a)
Only the two shared strings change (xl/sharedStrings.xml); every other part
of the workbook is byte-for-byte the same, no cell moves, and the version
stays 27. The bundled copy is the same file (template_sync passes;
editor_roundtrip and docs_links_check pass).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -629,7 +629,7 @@
     <t>* piezometric line 2 is only required for rapid drawdown analysis</t>
   </si>
   <si>
-    <t>Type optons</t>
+    <t>Type options</t>
   </si>
   <si>
     <t>True piezometric line: u = γw × vertical distance below the line (static head).</t>
@@ -638,7 +638,7 @@
     <t>phreatic</t>
   </si>
   <si>
-    <t xml:space="preserve"> Phreatic surface: static head reduced by cos² of the line's slope.</t>
+    <t>Phreatic surface: static head reduced by cos² of the line's slope.</t>
   </si>
   <si>
     <t>#</t>

</xml_diff>